<commit_message>
Add AI clinic integration: API, voice assistant, admin console
Adds the full AI integration layer so an external voice/chat assistant
(clinic-ai-assistant) can book appointments, check doctor schedules,
verify patients via OTP, and deliver reports through a scoped, audited
HTTP API, plus the admin console to configure doctors/locations/schedule
rules and telephony/voice receptionist support.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/billingwebapp/reports.xlsx
+++ b/billingwebapp/reports.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G123"/>
+  <dimension ref="A1:G134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4679,6 +4679,391 @@
         </is>
       </c>
     </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>INV-2026-1123</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>MR.SUSHIL DHADICH</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>7600019318</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>20-02-2026</t>
+        </is>
+      </c>
+      <c r="E124" t="n">
+        <v>1432.852</v>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>INV-2026-1124</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>MEERA DEVI</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>9784805340</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>20-02-2026</t>
+        </is>
+      </c>
+      <c r="E125" t="n">
+        <v>949.5989999999999</v>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>INV-2026-1125</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>MRS PINKY NAMA</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>9314171719</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>20-02-2026</t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>725.337</v>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>INV-2026-1126</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>VISHNU SINGH</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>9903023559</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>21-02-2026</t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>13884.284</v>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>INV-2026-1127</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>SHYAM KUMAR PAREEK</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>9828148228</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>21-02-2026</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>158.805</v>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>INV-2026-1128</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>DIVYA JOSHI</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>6376623725</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>23-02-2026</t>
+        </is>
+      </c>
+      <c r="E129" t="n">
+        <v>700.182</v>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>INV-2026-1129</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>VIJAY KHATRI</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>9950202448</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>23-02-2026</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>597.924</v>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>INV-2026-1130</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>SANSKRITI CHATURVEDI</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>797652057</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>23-02-2026</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>1494.126</v>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>INV-2026-1131</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>PURNIMA THANVI</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>9414141120</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>23-02-2026</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>548.424</v>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>INV-2026-1132</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>DR VIKAS JHANWAR</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>9887098702</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>23-02-2026</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>12541.52</v>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>INV-2026-1133</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>DR. MEGHA BHATI</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>9887003964</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>23-02-2026</t>
+        </is>
+      </c>
+      <c r="E134" t="n">
+        <v>779</v>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>